<commit_message>
Báo cáo tuần 7
</commit_message>
<xml_diff>
--- a/reports/week7.xlsx
+++ b/reports/week7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATN_NGUYEN_CHI_THANH\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD11A6F-4AAE-4C64-AC90-86529C2D2F70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E25999-C0B4-4099-A12A-F2AB438496EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F5557E33-1C4A-4FC1-8BEB-050DBAF2D33A}"/>
   </bookViews>
@@ -75,7 +75,7 @@
 Viết báo cáo tốt nghiệp					</t>
   </si>
   <si>
-    <t>Nghiên cứu tích hợp thêm ChatBotAI hỗ trợ tư vấn sản phẩm cần mua
+    <t xml:space="preserve">
 Fix các lỗi UX/UI gặp phải</t>
   </si>
 </sst>
@@ -148,15 +148,9 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -165,10 +159,16 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -512,128 +512,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="7">
         <v>7</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
     </row>
     <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="8">
         <v>45726</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
     </row>
     <row r="4" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="8">
         <v>45911</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
     </row>
     <row r="5" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
     </row>
     <row r="6" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="7">
         <v>191667</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
     </row>
     <row r="7" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
     </row>
     <row r="8" spans="1:8" ht="71" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" spans="1:8" ht="44.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>